<commit_message>
fix(doneledger): clarify founder fixture pack
</commit_message>
<xml_diff>
--- a/examples/doneledger/outputs/01a05d25-9174-7372-bf52-94f74ee90862/doneledger-founder-test-pack.xlsx
+++ b/examples/doneledger/outputs/01a05d25-9174-7372-bf52-94f74ee90862/doneledger-founder-test-pack.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rb086e7e8dbd94267"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Success 2 of 2" sheetId="2" r:id="R4fabf389c6054773"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions 3 of 5" sheetId="3" r:id="R95442e77950341b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invalid Total" sheetId="4" r:id="R341e6cfa40e84cb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Checklist" sheetId="5" r:id="R0278cf430ac04b9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R5120c7ad70de43b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Success 2 of 2" sheetId="2" r:id="R4af0962146e547a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mixed 3 Verified" sheetId="3" r:id="Rd84f29bf6afb4505"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invalid Total" sheetId="4" r:id="R9a074bae17a447b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Checklist" sheetId="5" r:id="R3b43c28f02a84e0d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -562,10 +562,10 @@
     </x:row>
     <x:row r="7" ht="36" customHeight="1">
       <x:c r="A7" s="18" t="str">
-        <x:v>Exception file</x:v>
+        <x:v>Mixed file</x:v>
       </x:c>
       <x:c r="B7" s="19" t="str">
-        <x:v>02-exceptions-3-of-5.csv → expect 3 verified, 1 FIELD_MISMATCH, 1 RECORD_MISSING</x:v>
+        <x:v>02-mixed-3-verified-of-5.csv → expect 3 verified, 1 FIELD_MISMATCH, 1 RECORD_MISSING</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="36" customHeight="1">
@@ -741,12 +741,12 @@
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Exceptions 3 of 5</x:v>
+        <x:v>Mixed 3 Verified</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Reference rows matching 02-exceptions-3-of-5.csv. Expected: 3 exact, 1 tax mismatch, 1 missing record.</x:v>
+        <x:v>Reference rows matching 02-mixed-3-verified-of-5.csv. Expected: 3 exact, 1 tax mismatch, 1 missing record.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -1178,10 +1178,10 @@
         <x:v>Exceptions</x:v>
       </x:c>
       <x:c r="C13" s="56" t="str">
-        <x:v>Upload/run 02-exceptions CSV</x:v>
+        <x:v>Upload/run 02-mixed CSV</x:v>
       </x:c>
       <x:c r="D13" s="56" t="str">
-        <x:v>3/5; mismatch + missing</x:v>
+        <x:v>3/5 verified; 2 exceptions</x:v>
       </x:c>
       <x:c r="E13" s="56" t="str">
         <x:v>Not Run</x:v>

</xml_diff>